<commit_message>
Update CSI - Report - [Intern's Name] - [Course Name] - [Step No].xlsx
minor edit the task name column title
</commit_message>
<xml_diff>
--- a/processes/Intern documents/CSI Templates/CSI - Report - [Intern's Name] - [Course Name] - [Step No].xlsx
+++ b/processes/Intern documents/CSI Templates/CSI - Report - [Intern's Name] - [Course Name] - [Step No].xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\asus\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\CS\cs-internship-spec\processes\Intern documents\CSI Templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC21B149-12F6-4B6A-99CB-103598858FF8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA50B851-F790-477D-B9C4-CD951194A8C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1125" yWindow="-120" windowWidth="19485" windowHeight="11760" xr2:uid="{55D2CF79-F578-4682-9360-5CC36F01DFB8}"/>
   </bookViews>
@@ -60,12 +60,6 @@
     <t>چه جلساتی شرکت کرده‌اید</t>
   </si>
   <si>
-    <t>استادی آیتم یا تسک</t>
-  </si>
-  <si>
-    <t>لینک پست</t>
-  </si>
-  <si>
     <t>به درصد (نمونه ۷۰%)</t>
   </si>
   <si>
@@ -136,6 +130,12 @@
   </si>
   <si>
     <t>بصورت توصیفی بگویید که روی چه مواردی کار کردید. این کارها چقدر  زمان می‌برند و در حین انجام با چه مشاهدات و کشفیاتی در مورد آن مسائل فنی روبرو شدید.</t>
+  </si>
+  <si>
+    <t>شماره و عنوان استادی آیتم یا تسک را مطابق شرح استپ بنویسید</t>
+  </si>
+  <si>
+    <t>لینک پست مربوط به هر تسک یا آیتم</t>
   </si>
 </sst>
 </file>
@@ -375,7 +375,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="48">
+  <cellXfs count="46">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -418,26 +418,59 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" indent="4"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" indent="4"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" indent="4"/>
-    </xf>
     <xf numFmtId="164" fontId="3" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" indent="4"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -448,71 +481,32 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" indent="4"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" indent="4"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" indent="4"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="right" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" indent="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -865,73 +859,79 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" s="1" customFormat="1" ht="26.25" x14ac:dyDescent="0.2">
-      <c r="A1" s="21" t="s">
-        <v>11</v>
-      </c>
-      <c r="B1" s="22"/>
-      <c r="C1" s="29" t="s">
+      <c r="A1" s="20" t="s">
+        <v>9</v>
+      </c>
+      <c r="B1" s="21"/>
+      <c r="C1" s="44" t="s">
+        <v>10</v>
+      </c>
+      <c r="D1" s="41"/>
+      <c r="E1" s="41"/>
+      <c r="F1" s="41"/>
+      <c r="G1" s="41"/>
+      <c r="H1" s="41"/>
+      <c r="I1" s="42"/>
+    </row>
+    <row r="2" spans="1:12" s="1" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="20" t="s">
+        <v>23</v>
+      </c>
+      <c r="B2" s="21"/>
+      <c r="C2" s="44" t="s">
+        <v>26</v>
+      </c>
+      <c r="D2" s="41"/>
+      <c r="E2" s="41"/>
+      <c r="F2" s="41"/>
+      <c r="G2" s="41"/>
+      <c r="H2" s="41"/>
+      <c r="I2" s="42"/>
+    </row>
+    <row r="3" spans="1:12" s="1" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="20" t="s">
         <v>12</v>
       </c>
-      <c r="D1" s="30"/>
-      <c r="E1" s="30"/>
-      <c r="F1" s="30"/>
-      <c r="G1" s="30"/>
-      <c r="H1" s="30"/>
-      <c r="I1" s="31"/>
-    </row>
-    <row r="2" spans="1:12" s="1" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="21" t="s">
+      <c r="B3" s="21"/>
+      <c r="C3" s="44" t="s">
+        <v>27</v>
+      </c>
+      <c r="D3" s="41"/>
+      <c r="E3" s="41"/>
+      <c r="F3" s="41"/>
+      <c r="G3" s="41"/>
+      <c r="H3" s="41"/>
+      <c r="I3" s="42"/>
+    </row>
+    <row r="4" spans="1:12" s="1" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="20" t="s">
         <v>25</v>
       </c>
-      <c r="B2" s="22"/>
-      <c r="C2" s="16" t="s">
+      <c r="B4" s="21"/>
+      <c r="C4" s="44" t="s">
         <v>28</v>
       </c>
-      <c r="D2" s="17"/>
-      <c r="E2" s="17"/>
-      <c r="F2" s="17"/>
-      <c r="G2" s="17"/>
-      <c r="H2" s="17"/>
-      <c r="I2" s="18"/>
-    </row>
-    <row r="3" spans="1:12" s="1" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="21" t="s">
-        <v>14</v>
-      </c>
-      <c r="B3" s="22"/>
-      <c r="C3" s="29" t="s">
-        <v>29</v>
-      </c>
-      <c r="D3" s="30"/>
-      <c r="E3" s="30"/>
-      <c r="F3" s="30"/>
-      <c r="G3" s="30"/>
-      <c r="H3" s="30"/>
-      <c r="I3" s="31"/>
-    </row>
-    <row r="4" spans="1:12" s="1" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="21" t="s">
-        <v>27</v>
-      </c>
-      <c r="B4" s="22"/>
-      <c r="C4" s="16" t="s">
-        <v>30</v>
-      </c>
-      <c r="D4" s="17"/>
-      <c r="E4" s="17"/>
-      <c r="F4" s="17"/>
-      <c r="G4" s="17"/>
-      <c r="H4" s="17"/>
-      <c r="I4" s="18"/>
+      <c r="D4" s="41"/>
+      <c r="E4" s="41"/>
+      <c r="F4" s="41"/>
+      <c r="G4" s="41"/>
+      <c r="H4" s="41"/>
+      <c r="I4" s="42"/>
     </row>
     <row r="5" spans="1:12" s="1" customFormat="1" ht="26.25" x14ac:dyDescent="0.2">
-      <c r="A5" s="21" t="s">
-        <v>26</v>
-      </c>
-      <c r="B5" s="22"/>
-      <c r="C5" s="20">
+      <c r="A5" s="20" t="s">
+        <v>24</v>
+      </c>
+      <c r="B5" s="21"/>
+      <c r="C5" s="45">
         <v>7</v>
       </c>
+      <c r="D5" s="43"/>
+      <c r="E5" s="43"/>
+      <c r="F5" s="43"/>
+      <c r="G5" s="43"/>
+      <c r="H5" s="43"/>
+      <c r="I5" s="43"/>
     </row>
     <row r="6" spans="1:12" s="5" customFormat="1" ht="52.5" x14ac:dyDescent="0.2">
       <c r="A6" s="8" t="s">
@@ -946,12 +946,12 @@
       <c r="D6" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="E6" s="41" t="s">
+      <c r="E6" s="40" t="s">
         <v>2</v>
       </c>
-      <c r="F6" s="41"/>
+      <c r="F6" s="40"/>
       <c r="G6" s="9" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="H6" s="8" t="s">
         <v>7</v>
@@ -967,546 +967,579 @@
       <c r="A7" s="10"/>
       <c r="B7" s="10"/>
       <c r="C7" s="11" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="D7" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="E7" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="F7" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="E7" s="10" t="s">
+      <c r="G7" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="H7" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="I7" s="10" t="s">
         <v>8</v>
-      </c>
-      <c r="F7" s="10" t="s">
-        <v>9</v>
-      </c>
-      <c r="G7" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="H7" s="11" t="s">
-        <v>17</v>
-      </c>
-      <c r="I7" s="10" t="s">
-        <v>10</v>
       </c>
       <c r="J7" s="13"/>
       <c r="K7" s="13"/>
       <c r="L7" s="13"/>
     </row>
     <row r="8" spans="1:12" s="3" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="33" t="s">
+      <c r="A8" s="23" t="s">
         <v>5</v>
       </c>
-      <c r="B8" s="33" t="s">
-        <v>31</v>
-      </c>
-      <c r="C8" s="42">
+      <c r="B8" s="23" t="s">
+        <v>29</v>
+      </c>
+      <c r="C8" s="26">
         <v>0</v>
       </c>
-      <c r="D8" s="39"/>
+      <c r="D8" s="29"/>
       <c r="E8" s="7"/>
-      <c r="F8" s="45"/>
-      <c r="G8" s="25"/>
+      <c r="F8" s="17"/>
+      <c r="G8" s="36"/>
       <c r="H8" s="7"/>
-      <c r="I8" s="33"/>
+      <c r="I8" s="23"/>
     </row>
     <row r="9" spans="1:12" s="3" customFormat="1" ht="21.75" x14ac:dyDescent="0.2">
-      <c r="A9" s="33"/>
-      <c r="B9" s="33"/>
-      <c r="C9" s="42"/>
-      <c r="D9" s="39"/>
+      <c r="A9" s="23"/>
+      <c r="B9" s="23"/>
+      <c r="C9" s="26"/>
+      <c r="D9" s="29"/>
       <c r="E9" s="7"/>
-      <c r="F9" s="45"/>
-      <c r="G9" s="26"/>
+      <c r="F9" s="17"/>
+      <c r="G9" s="32"/>
       <c r="H9" s="7"/>
-      <c r="I9" s="33"/>
+      <c r="I9" s="23"/>
     </row>
     <row r="10" spans="1:12" s="3" customFormat="1" ht="21.75" x14ac:dyDescent="0.2">
-      <c r="A10" s="33"/>
-      <c r="B10" s="33"/>
-      <c r="C10" s="42"/>
-      <c r="D10" s="39"/>
+      <c r="A10" s="23"/>
+      <c r="B10" s="23"/>
+      <c r="C10" s="26"/>
+      <c r="D10" s="29"/>
       <c r="E10" s="7"/>
-      <c r="F10" s="45"/>
-      <c r="G10" s="26"/>
+      <c r="F10" s="17"/>
+      <c r="G10" s="32"/>
       <c r="H10" s="7"/>
-      <c r="I10" s="33"/>
+      <c r="I10" s="23"/>
     </row>
     <row r="11" spans="1:12" s="3" customFormat="1" ht="21.75" x14ac:dyDescent="0.2">
-      <c r="A11" s="33"/>
-      <c r="B11" s="33"/>
-      <c r="C11" s="42"/>
-      <c r="D11" s="39"/>
+      <c r="A11" s="23"/>
+      <c r="B11" s="23"/>
+      <c r="C11" s="26"/>
+      <c r="D11" s="29"/>
       <c r="E11" s="7"/>
-      <c r="F11" s="45"/>
-      <c r="G11" s="26"/>
+      <c r="F11" s="17"/>
+      <c r="G11" s="32"/>
       <c r="H11" s="7"/>
-      <c r="I11" s="33"/>
+      <c r="I11" s="23"/>
     </row>
     <row r="12" spans="1:12" s="3" customFormat="1" ht="21.75" x14ac:dyDescent="0.2">
-      <c r="A12" s="33"/>
-      <c r="B12" s="33"/>
-      <c r="C12" s="42"/>
-      <c r="D12" s="39"/>
+      <c r="A12" s="23"/>
+      <c r="B12" s="23"/>
+      <c r="C12" s="26"/>
+      <c r="D12" s="29"/>
       <c r="E12" s="7"/>
-      <c r="F12" s="45"/>
-      <c r="G12" s="26"/>
+      <c r="F12" s="17"/>
+      <c r="G12" s="32"/>
       <c r="H12" s="7"/>
-      <c r="I12" s="33"/>
+      <c r="I12" s="23"/>
     </row>
     <row r="13" spans="1:12" s="3" customFormat="1" ht="28.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="34"/>
-      <c r="B13" s="34"/>
-      <c r="C13" s="43"/>
-      <c r="D13" s="40"/>
+      <c r="A13" s="24"/>
+      <c r="B13" s="24"/>
+      <c r="C13" s="27"/>
+      <c r="D13" s="30"/>
       <c r="E13" s="14"/>
-      <c r="F13" s="46"/>
-      <c r="G13" s="27"/>
+      <c r="F13" s="18"/>
+      <c r="G13" s="33"/>
       <c r="H13" s="14"/>
-      <c r="I13" s="34"/>
+      <c r="I13" s="24"/>
     </row>
     <row r="14" spans="1:12" s="3" customFormat="1" ht="27" customHeight="1" thickTop="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="32" t="s">
-        <v>13</v>
-      </c>
-      <c r="B14" s="32" t="s">
-        <v>31</v>
-      </c>
-      <c r="C14" s="35">
+      <c r="A14" s="22" t="s">
+        <v>11</v>
+      </c>
+      <c r="B14" s="22" t="s">
+        <v>29</v>
+      </c>
+      <c r="C14" s="37">
         <v>0</v>
       </c>
-      <c r="D14" s="38"/>
+      <c r="D14" s="28"/>
       <c r="E14" s="15"/>
-      <c r="F14" s="47"/>
-      <c r="G14" s="28"/>
+      <c r="F14" s="19"/>
+      <c r="G14" s="31"/>
       <c r="H14" s="15"/>
-      <c r="I14" s="32"/>
+      <c r="I14" s="22"/>
     </row>
     <row r="15" spans="1:12" s="3" customFormat="1" ht="21.75" x14ac:dyDescent="0.2">
-      <c r="A15" s="33"/>
-      <c r="B15" s="33"/>
-      <c r="C15" s="36"/>
-      <c r="D15" s="39"/>
+      <c r="A15" s="23"/>
+      <c r="B15" s="23"/>
+      <c r="C15" s="38"/>
+      <c r="D15" s="29"/>
       <c r="E15" s="7"/>
-      <c r="F15" s="45"/>
-      <c r="G15" s="26"/>
+      <c r="F15" s="17"/>
+      <c r="G15" s="32"/>
       <c r="H15" s="7"/>
-      <c r="I15" s="33"/>
+      <c r="I15" s="23"/>
     </row>
     <row r="16" spans="1:12" s="3" customFormat="1" ht="21.75" x14ac:dyDescent="0.2">
-      <c r="A16" s="33"/>
-      <c r="B16" s="33"/>
-      <c r="C16" s="36"/>
-      <c r="D16" s="39"/>
+      <c r="A16" s="23"/>
+      <c r="B16" s="23"/>
+      <c r="C16" s="38"/>
+      <c r="D16" s="29"/>
       <c r="E16" s="7"/>
-      <c r="F16" s="45"/>
-      <c r="G16" s="26"/>
+      <c r="F16" s="17"/>
+      <c r="G16" s="32"/>
       <c r="H16" s="7"/>
-      <c r="I16" s="33"/>
+      <c r="I16" s="23"/>
     </row>
     <row r="17" spans="1:9" s="3" customFormat="1" ht="21.75" x14ac:dyDescent="0.2">
-      <c r="A17" s="33"/>
-      <c r="B17" s="33"/>
-      <c r="C17" s="36"/>
-      <c r="D17" s="39"/>
+      <c r="A17" s="23"/>
+      <c r="B17" s="23"/>
+      <c r="C17" s="38"/>
+      <c r="D17" s="29"/>
       <c r="E17" s="7"/>
-      <c r="F17" s="45"/>
-      <c r="G17" s="26"/>
+      <c r="F17" s="17"/>
+      <c r="G17" s="32"/>
       <c r="H17" s="7"/>
-      <c r="I17" s="33"/>
+      <c r="I17" s="23"/>
     </row>
     <row r="18" spans="1:9" s="3" customFormat="1" ht="21.75" x14ac:dyDescent="0.2">
-      <c r="A18" s="33"/>
-      <c r="B18" s="33"/>
-      <c r="C18" s="36"/>
-      <c r="D18" s="39"/>
+      <c r="A18" s="23"/>
+      <c r="B18" s="23"/>
+      <c r="C18" s="38"/>
+      <c r="D18" s="29"/>
       <c r="E18" s="7"/>
-      <c r="F18" s="45"/>
-      <c r="G18" s="26"/>
+      <c r="F18" s="17"/>
+      <c r="G18" s="32"/>
       <c r="H18" s="7"/>
-      <c r="I18" s="33"/>
+      <c r="I18" s="23"/>
     </row>
     <row r="19" spans="1:9" s="3" customFormat="1" ht="28.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="34"/>
-      <c r="B19" s="34"/>
-      <c r="C19" s="37"/>
-      <c r="D19" s="40"/>
+      <c r="A19" s="24"/>
+      <c r="B19" s="24"/>
+      <c r="C19" s="39"/>
+      <c r="D19" s="30"/>
       <c r="E19" s="14"/>
-      <c r="F19" s="46"/>
-      <c r="G19" s="27"/>
+      <c r="F19" s="18"/>
+      <c r="G19" s="33"/>
       <c r="H19" s="14"/>
-      <c r="I19" s="34"/>
+      <c r="I19" s="24"/>
     </row>
     <row r="20" spans="1:9" s="3" customFormat="1" ht="22.5" thickTop="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="32" t="s">
+      <c r="A20" s="22" t="s">
+        <v>16</v>
+      </c>
+      <c r="B20" s="22" t="s">
+        <v>29</v>
+      </c>
+      <c r="C20" s="25">
+        <v>0</v>
+      </c>
+      <c r="D20" s="28"/>
+      <c r="E20" s="15"/>
+      <c r="F20" s="19"/>
+      <c r="G20" s="31"/>
+      <c r="H20" s="15"/>
+      <c r="I20" s="22"/>
+    </row>
+    <row r="21" spans="1:9" s="3" customFormat="1" ht="21.75" x14ac:dyDescent="0.2">
+      <c r="A21" s="23"/>
+      <c r="B21" s="23"/>
+      <c r="C21" s="26"/>
+      <c r="D21" s="29"/>
+      <c r="E21" s="7"/>
+      <c r="F21" s="17"/>
+      <c r="G21" s="32"/>
+      <c r="H21" s="7"/>
+      <c r="I21" s="23"/>
+    </row>
+    <row r="22" spans="1:9" s="3" customFormat="1" ht="21.75" x14ac:dyDescent="0.2">
+      <c r="A22" s="23"/>
+      <c r="B22" s="23"/>
+      <c r="C22" s="26"/>
+      <c r="D22" s="29"/>
+      <c r="E22" s="7"/>
+      <c r="F22" s="17"/>
+      <c r="G22" s="32"/>
+      <c r="H22" s="7"/>
+      <c r="I22" s="23"/>
+    </row>
+    <row r="23" spans="1:9" s="3" customFormat="1" ht="21.75" x14ac:dyDescent="0.2">
+      <c r="A23" s="23"/>
+      <c r="B23" s="23"/>
+      <c r="C23" s="26"/>
+      <c r="D23" s="29"/>
+      <c r="E23" s="7"/>
+      <c r="F23" s="17"/>
+      <c r="G23" s="32"/>
+      <c r="H23" s="7"/>
+      <c r="I23" s="23"/>
+    </row>
+    <row r="24" spans="1:9" s="3" customFormat="1" ht="21.75" x14ac:dyDescent="0.2">
+      <c r="A24" s="23"/>
+      <c r="B24" s="23"/>
+      <c r="C24" s="26"/>
+      <c r="D24" s="29"/>
+      <c r="E24" s="7"/>
+      <c r="F24" s="17"/>
+      <c r="G24" s="32"/>
+      <c r="H24" s="7"/>
+      <c r="I24" s="23"/>
+    </row>
+    <row r="25" spans="1:9" s="3" customFormat="1" ht="22.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="24"/>
+      <c r="B25" s="24"/>
+      <c r="C25" s="27"/>
+      <c r="D25" s="30"/>
+      <c r="E25" s="14"/>
+      <c r="F25" s="18"/>
+      <c r="G25" s="33"/>
+      <c r="H25" s="14"/>
+      <c r="I25" s="24"/>
+    </row>
+    <row r="26" spans="1:9" s="4" customFormat="1" ht="22.5" thickTop="1" x14ac:dyDescent="0.5">
+      <c r="A26" s="22" t="s">
+        <v>17</v>
+      </c>
+      <c r="B26" s="22" t="s">
+        <v>29</v>
+      </c>
+      <c r="C26" s="25">
+        <v>0</v>
+      </c>
+      <c r="D26" s="28"/>
+      <c r="E26" s="15"/>
+      <c r="F26" s="19"/>
+      <c r="G26" s="31"/>
+      <c r="H26" s="15"/>
+      <c r="I26" s="22"/>
+    </row>
+    <row r="27" spans="1:9" s="4" customFormat="1" ht="21.75" x14ac:dyDescent="0.5">
+      <c r="A27" s="23"/>
+      <c r="B27" s="23"/>
+      <c r="C27" s="26"/>
+      <c r="D27" s="29"/>
+      <c r="E27" s="7"/>
+      <c r="F27" s="17"/>
+      <c r="G27" s="32"/>
+      <c r="H27" s="7"/>
+      <c r="I27" s="23"/>
+    </row>
+    <row r="28" spans="1:9" s="2" customFormat="1" ht="21.75" x14ac:dyDescent="0.6">
+      <c r="A28" s="23"/>
+      <c r="B28" s="23"/>
+      <c r="C28" s="26"/>
+      <c r="D28" s="29"/>
+      <c r="E28" s="7"/>
+      <c r="F28" s="17"/>
+      <c r="G28" s="32"/>
+      <c r="H28" s="7"/>
+      <c r="I28" s="23"/>
+    </row>
+    <row r="29" spans="1:9" s="2" customFormat="1" ht="21.75" x14ac:dyDescent="0.6">
+      <c r="A29" s="23"/>
+      <c r="B29" s="23"/>
+      <c r="C29" s="26"/>
+      <c r="D29" s="29"/>
+      <c r="E29" s="7"/>
+      <c r="F29" s="17"/>
+      <c r="G29" s="32"/>
+      <c r="H29" s="7"/>
+      <c r="I29" s="23"/>
+    </row>
+    <row r="30" spans="1:9" s="2" customFormat="1" ht="21.75" x14ac:dyDescent="0.6">
+      <c r="A30" s="23"/>
+      <c r="B30" s="23"/>
+      <c r="C30" s="26"/>
+      <c r="D30" s="29"/>
+      <c r="E30" s="7"/>
+      <c r="F30" s="17"/>
+      <c r="G30" s="32"/>
+      <c r="H30" s="7"/>
+      <c r="I30" s="23"/>
+    </row>
+    <row r="31" spans="1:9" s="2" customFormat="1" ht="22.5" thickBot="1" x14ac:dyDescent="0.65">
+      <c r="A31" s="24"/>
+      <c r="B31" s="24"/>
+      <c r="C31" s="27"/>
+      <c r="D31" s="30"/>
+      <c r="E31" s="14"/>
+      <c r="F31" s="18"/>
+      <c r="G31" s="33"/>
+      <c r="H31" s="14"/>
+      <c r="I31" s="24"/>
+    </row>
+    <row r="32" spans="1:9" ht="22.5" thickTop="1" x14ac:dyDescent="0.2">
+      <c r="A32" s="22" t="s">
         <v>18</v>
       </c>
-      <c r="B20" s="32" t="s">
-        <v>31</v>
-      </c>
-      <c r="C20" s="44">
+      <c r="B32" s="22" t="s">
+        <v>30</v>
+      </c>
+      <c r="C32" s="25">
         <v>0</v>
       </c>
-      <c r="D20" s="38"/>
-      <c r="E20" s="15"/>
-      <c r="F20" s="47"/>
-      <c r="G20" s="28"/>
-      <c r="H20" s="15"/>
-      <c r="I20" s="32"/>
-    </row>
-    <row r="21" spans="1:9" s="3" customFormat="1" ht="21.75" x14ac:dyDescent="0.2">
-      <c r="A21" s="33"/>
-      <c r="B21" s="33"/>
-      <c r="C21" s="42"/>
-      <c r="D21" s="39"/>
-      <c r="E21" s="7"/>
-      <c r="F21" s="45"/>
-      <c r="G21" s="26"/>
-      <c r="H21" s="7"/>
-      <c r="I21" s="33"/>
-    </row>
-    <row r="22" spans="1:9" s="3" customFormat="1" ht="21.75" x14ac:dyDescent="0.2">
-      <c r="A22" s="33"/>
-      <c r="B22" s="33"/>
-      <c r="C22" s="42"/>
-      <c r="D22" s="39"/>
-      <c r="E22" s="7"/>
-      <c r="F22" s="45"/>
-      <c r="G22" s="26"/>
-      <c r="H22" s="7"/>
-      <c r="I22" s="33"/>
-    </row>
-    <row r="23" spans="1:9" s="3" customFormat="1" ht="21.75" x14ac:dyDescent="0.2">
-      <c r="A23" s="33"/>
-      <c r="B23" s="33"/>
-      <c r="C23" s="42"/>
-      <c r="D23" s="39"/>
-      <c r="E23" s="7"/>
-      <c r="F23" s="45"/>
-      <c r="G23" s="26"/>
-      <c r="H23" s="7"/>
-      <c r="I23" s="33"/>
-    </row>
-    <row r="24" spans="1:9" s="3" customFormat="1" ht="21.75" x14ac:dyDescent="0.2">
-      <c r="A24" s="33"/>
-      <c r="B24" s="33"/>
-      <c r="C24" s="42"/>
-      <c r="D24" s="39"/>
-      <c r="E24" s="7"/>
-      <c r="F24" s="45"/>
-      <c r="G24" s="26"/>
-      <c r="H24" s="7"/>
-      <c r="I24" s="33"/>
-    </row>
-    <row r="25" spans="1:9" s="3" customFormat="1" ht="22.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="34"/>
-      <c r="B25" s="34"/>
-      <c r="C25" s="43"/>
-      <c r="D25" s="40"/>
-      <c r="E25" s="14"/>
-      <c r="F25" s="46"/>
-      <c r="G25" s="27"/>
-      <c r="H25" s="14"/>
-      <c r="I25" s="34"/>
-    </row>
-    <row r="26" spans="1:9" s="4" customFormat="1" ht="22.5" thickTop="1" x14ac:dyDescent="0.5">
-      <c r="A26" s="32" t="s">
+      <c r="D32" s="28"/>
+      <c r="E32" s="15"/>
+      <c r="F32" s="19"/>
+      <c r="G32" s="31"/>
+      <c r="H32" s="15"/>
+      <c r="I32" s="22"/>
+    </row>
+    <row r="33" spans="1:9" ht="21.75" x14ac:dyDescent="0.2">
+      <c r="A33" s="23"/>
+      <c r="B33" s="23"/>
+      <c r="C33" s="26"/>
+      <c r="D33" s="29"/>
+      <c r="E33" s="7"/>
+      <c r="F33" s="17"/>
+      <c r="G33" s="32"/>
+      <c r="H33" s="7"/>
+      <c r="I33" s="23"/>
+    </row>
+    <row r="34" spans="1:9" ht="21.75" x14ac:dyDescent="0.2">
+      <c r="A34" s="23"/>
+      <c r="B34" s="23"/>
+      <c r="C34" s="26"/>
+      <c r="D34" s="29"/>
+      <c r="E34" s="7"/>
+      <c r="F34" s="17"/>
+      <c r="G34" s="32"/>
+      <c r="H34" s="7"/>
+      <c r="I34" s="23"/>
+    </row>
+    <row r="35" spans="1:9" ht="21.75" x14ac:dyDescent="0.2">
+      <c r="A35" s="23"/>
+      <c r="B35" s="23"/>
+      <c r="C35" s="26"/>
+      <c r="D35" s="29"/>
+      <c r="E35" s="7"/>
+      <c r="F35" s="17"/>
+      <c r="G35" s="32"/>
+      <c r="H35" s="7"/>
+      <c r="I35" s="23"/>
+    </row>
+    <row r="36" spans="1:9" ht="21.75" x14ac:dyDescent="0.2">
+      <c r="A36" s="23"/>
+      <c r="B36" s="23"/>
+      <c r="C36" s="26"/>
+      <c r="D36" s="29"/>
+      <c r="E36" s="7"/>
+      <c r="F36" s="17"/>
+      <c r="G36" s="32"/>
+      <c r="H36" s="7"/>
+      <c r="I36" s="23"/>
+    </row>
+    <row r="37" spans="1:9" ht="22.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A37" s="24"/>
+      <c r="B37" s="24"/>
+      <c r="C37" s="27"/>
+      <c r="D37" s="30"/>
+      <c r="E37" s="14"/>
+      <c r="F37" s="18"/>
+      <c r="G37" s="33"/>
+      <c r="H37" s="14"/>
+      <c r="I37" s="24"/>
+    </row>
+    <row r="38" spans="1:9" ht="22.5" thickTop="1" x14ac:dyDescent="0.2">
+      <c r="A38" s="22" t="s">
         <v>19</v>
       </c>
-      <c r="B26" s="32" t="s">
-        <v>31</v>
-      </c>
-      <c r="C26" s="44">
+      <c r="B38" s="22" t="s">
+        <v>29</v>
+      </c>
+      <c r="C38" s="25">
         <v>0</v>
       </c>
-      <c r="D26" s="38"/>
-      <c r="E26" s="15"/>
-      <c r="F26" s="47"/>
-      <c r="G26" s="28"/>
-      <c r="H26" s="15"/>
-      <c r="I26" s="32"/>
-    </row>
-    <row r="27" spans="1:9" s="4" customFormat="1" ht="21.75" x14ac:dyDescent="0.5">
-      <c r="A27" s="33"/>
-      <c r="B27" s="33"/>
-      <c r="C27" s="42"/>
-      <c r="D27" s="39"/>
-      <c r="E27" s="7"/>
-      <c r="F27" s="45"/>
-      <c r="G27" s="26"/>
-      <c r="H27" s="7"/>
-      <c r="I27" s="33"/>
-    </row>
-    <row r="28" spans="1:9" s="2" customFormat="1" ht="21.75" x14ac:dyDescent="0.6">
-      <c r="A28" s="33"/>
-      <c r="B28" s="33"/>
-      <c r="C28" s="42"/>
-      <c r="D28" s="39"/>
-      <c r="E28" s="7"/>
-      <c r="F28" s="45"/>
-      <c r="G28" s="26"/>
-      <c r="H28" s="7"/>
-      <c r="I28" s="33"/>
-    </row>
-    <row r="29" spans="1:9" s="2" customFormat="1" ht="21.75" x14ac:dyDescent="0.6">
-      <c r="A29" s="33"/>
-      <c r="B29" s="33"/>
-      <c r="C29" s="42"/>
-      <c r="D29" s="39"/>
-      <c r="E29" s="7"/>
-      <c r="F29" s="45"/>
-      <c r="G29" s="26"/>
-      <c r="H29" s="7"/>
-      <c r="I29" s="33"/>
-    </row>
-    <row r="30" spans="1:9" s="2" customFormat="1" ht="21.75" x14ac:dyDescent="0.6">
-      <c r="A30" s="33"/>
-      <c r="B30" s="33"/>
-      <c r="C30" s="42"/>
-      <c r="D30" s="39"/>
-      <c r="E30" s="7"/>
-      <c r="F30" s="45"/>
-      <c r="G30" s="26"/>
-      <c r="H30" s="7"/>
-      <c r="I30" s="33"/>
-    </row>
-    <row r="31" spans="1:9" s="2" customFormat="1" ht="22.5" thickBot="1" x14ac:dyDescent="0.65">
-      <c r="A31" s="34"/>
-      <c r="B31" s="34"/>
-      <c r="C31" s="43"/>
-      <c r="D31" s="40"/>
-      <c r="E31" s="14"/>
-      <c r="F31" s="46"/>
-      <c r="G31" s="27"/>
-      <c r="H31" s="14"/>
-      <c r="I31" s="34"/>
-    </row>
-    <row r="32" spans="1:9" ht="22.5" thickTop="1" x14ac:dyDescent="0.2">
-      <c r="A32" s="32" t="s">
+      <c r="D38" s="28"/>
+      <c r="E38" s="15"/>
+      <c r="F38" s="19"/>
+      <c r="G38" s="31"/>
+      <c r="H38" s="15"/>
+      <c r="I38" s="22"/>
+    </row>
+    <row r="39" spans="1:9" ht="21.75" x14ac:dyDescent="0.2">
+      <c r="A39" s="23"/>
+      <c r="B39" s="23"/>
+      <c r="C39" s="26"/>
+      <c r="D39" s="29"/>
+      <c r="E39" s="7"/>
+      <c r="F39" s="17"/>
+      <c r="G39" s="32"/>
+      <c r="H39" s="7"/>
+      <c r="I39" s="23"/>
+    </row>
+    <row r="40" spans="1:9" ht="21.75" x14ac:dyDescent="0.2">
+      <c r="A40" s="23"/>
+      <c r="B40" s="23"/>
+      <c r="C40" s="26"/>
+      <c r="D40" s="29"/>
+      <c r="E40" s="7"/>
+      <c r="F40" s="17"/>
+      <c r="G40" s="32"/>
+      <c r="H40" s="7"/>
+      <c r="I40" s="23"/>
+    </row>
+    <row r="41" spans="1:9" ht="21.75" x14ac:dyDescent="0.2">
+      <c r="A41" s="23"/>
+      <c r="B41" s="23"/>
+      <c r="C41" s="26"/>
+      <c r="D41" s="29"/>
+      <c r="E41" s="7"/>
+      <c r="F41" s="17"/>
+      <c r="G41" s="32"/>
+      <c r="H41" s="7"/>
+      <c r="I41" s="23"/>
+    </row>
+    <row r="42" spans="1:9" ht="21.75" x14ac:dyDescent="0.2">
+      <c r="A42" s="23"/>
+      <c r="B42" s="23"/>
+      <c r="C42" s="26"/>
+      <c r="D42" s="29"/>
+      <c r="E42" s="7"/>
+      <c r="F42" s="17"/>
+      <c r="G42" s="32"/>
+      <c r="H42" s="7"/>
+      <c r="I42" s="23"/>
+    </row>
+    <row r="43" spans="1:9" ht="22.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A43" s="24"/>
+      <c r="B43" s="24"/>
+      <c r="C43" s="27"/>
+      <c r="D43" s="30"/>
+      <c r="E43" s="14"/>
+      <c r="F43" s="18"/>
+      <c r="G43" s="33"/>
+      <c r="H43" s="14"/>
+      <c r="I43" s="24"/>
+    </row>
+    <row r="44" spans="1:9" ht="22.5" thickTop="1" x14ac:dyDescent="0.2">
+      <c r="A44" s="22" t="s">
         <v>20</v>
       </c>
-      <c r="B32" s="32" t="s">
-        <v>32</v>
-      </c>
-      <c r="C32" s="44">
+      <c r="B44" s="22" t="s">
+        <v>29</v>
+      </c>
+      <c r="C44" s="25">
         <v>0</v>
       </c>
-      <c r="D32" s="38"/>
-      <c r="E32" s="15"/>
-      <c r="F32" s="47"/>
-      <c r="G32" s="28"/>
-      <c r="H32" s="15"/>
-      <c r="I32" s="32"/>
-    </row>
-    <row r="33" spans="1:9" ht="21.75" x14ac:dyDescent="0.2">
-      <c r="A33" s="33"/>
-      <c r="B33" s="33"/>
-      <c r="C33" s="42"/>
-      <c r="D33" s="39"/>
-      <c r="E33" s="7"/>
-      <c r="F33" s="45"/>
-      <c r="G33" s="26"/>
-      <c r="H33" s="7"/>
-      <c r="I33" s="33"/>
-    </row>
-    <row r="34" spans="1:9" ht="21.75" x14ac:dyDescent="0.2">
-      <c r="A34" s="33"/>
-      <c r="B34" s="33"/>
-      <c r="C34" s="42"/>
-      <c r="D34" s="39"/>
-      <c r="E34" s="7"/>
-      <c r="F34" s="45"/>
-      <c r="G34" s="26"/>
-      <c r="H34" s="7"/>
-      <c r="I34" s="33"/>
-    </row>
-    <row r="35" spans="1:9" ht="21.75" x14ac:dyDescent="0.2">
-      <c r="A35" s="33"/>
-      <c r="B35" s="33"/>
-      <c r="C35" s="42"/>
-      <c r="D35" s="39"/>
-      <c r="E35" s="7"/>
-      <c r="F35" s="45"/>
-      <c r="G35" s="26"/>
-      <c r="H35" s="7"/>
-      <c r="I35" s="33"/>
-    </row>
-    <row r="36" spans="1:9" ht="21.75" x14ac:dyDescent="0.2">
-      <c r="A36" s="33"/>
-      <c r="B36" s="33"/>
-      <c r="C36" s="42"/>
-      <c r="D36" s="39"/>
-      <c r="E36" s="7"/>
-      <c r="F36" s="45"/>
-      <c r="G36" s="26"/>
-      <c r="H36" s="7"/>
-      <c r="I36" s="33"/>
-    </row>
-    <row r="37" spans="1:9" ht="22.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="34"/>
-      <c r="B37" s="34"/>
-      <c r="C37" s="43"/>
-      <c r="D37" s="40"/>
-      <c r="E37" s="14"/>
-      <c r="F37" s="46"/>
-      <c r="G37" s="27"/>
-      <c r="H37" s="14"/>
-      <c r="I37" s="34"/>
-    </row>
-    <row r="38" spans="1:9" ht="22.5" thickTop="1" x14ac:dyDescent="0.2">
-      <c r="A38" s="32" t="s">
+      <c r="D44" s="28"/>
+      <c r="E44" s="15"/>
+      <c r="F44" s="19"/>
+      <c r="G44" s="31"/>
+      <c r="H44" s="15"/>
+      <c r="I44" s="22"/>
+    </row>
+    <row r="45" spans="1:9" ht="21.75" x14ac:dyDescent="0.2">
+      <c r="A45" s="23"/>
+      <c r="B45" s="23"/>
+      <c r="C45" s="26"/>
+      <c r="D45" s="29"/>
+      <c r="E45" s="7"/>
+      <c r="F45" s="17"/>
+      <c r="G45" s="32"/>
+      <c r="H45" s="7"/>
+      <c r="I45" s="23"/>
+    </row>
+    <row r="46" spans="1:9" ht="21.75" x14ac:dyDescent="0.2">
+      <c r="A46" s="23"/>
+      <c r="B46" s="23"/>
+      <c r="C46" s="26"/>
+      <c r="D46" s="29"/>
+      <c r="E46" s="7"/>
+      <c r="F46" s="17"/>
+      <c r="G46" s="32"/>
+      <c r="H46" s="7"/>
+      <c r="I46" s="23"/>
+    </row>
+    <row r="47" spans="1:9" ht="21.75" x14ac:dyDescent="0.2">
+      <c r="A47" s="23"/>
+      <c r="B47" s="23"/>
+      <c r="C47" s="26"/>
+      <c r="D47" s="29"/>
+      <c r="E47" s="7"/>
+      <c r="F47" s="17"/>
+      <c r="G47" s="32"/>
+      <c r="H47" s="7"/>
+      <c r="I47" s="23"/>
+    </row>
+    <row r="48" spans="1:9" ht="21.75" x14ac:dyDescent="0.2">
+      <c r="A48" s="23"/>
+      <c r="B48" s="23"/>
+      <c r="C48" s="26"/>
+      <c r="D48" s="29"/>
+      <c r="E48" s="7"/>
+      <c r="F48" s="17"/>
+      <c r="G48" s="32"/>
+      <c r="H48" s="7"/>
+      <c r="I48" s="23"/>
+    </row>
+    <row r="49" spans="1:9" ht="22.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A49" s="24"/>
+      <c r="B49" s="24"/>
+      <c r="C49" s="27"/>
+      <c r="D49" s="30"/>
+      <c r="E49" s="14"/>
+      <c r="F49" s="18"/>
+      <c r="G49" s="33"/>
+      <c r="H49" s="14"/>
+      <c r="I49" s="24"/>
+    </row>
+    <row r="50" spans="1:9" ht="66.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.2">
+      <c r="A50" s="34" t="s">
         <v>21</v>
       </c>
-      <c r="B38" s="32" t="s">
-        <v>31</v>
-      </c>
-      <c r="C38" s="44">
-        <v>0</v>
-      </c>
-      <c r="D38" s="38"/>
-      <c r="E38" s="15"/>
-      <c r="F38" s="47"/>
-      <c r="G38" s="28"/>
-      <c r="H38" s="15"/>
-      <c r="I38" s="32"/>
-    </row>
-    <row r="39" spans="1:9" ht="21.75" x14ac:dyDescent="0.2">
-      <c r="A39" s="33"/>
-      <c r="B39" s="33"/>
-      <c r="C39" s="42"/>
-      <c r="D39" s="39"/>
-      <c r="E39" s="7"/>
-      <c r="F39" s="45"/>
-      <c r="G39" s="26"/>
-      <c r="H39" s="7"/>
-      <c r="I39" s="33"/>
-    </row>
-    <row r="40" spans="1:9" ht="21.75" x14ac:dyDescent="0.2">
-      <c r="A40" s="33"/>
-      <c r="B40" s="33"/>
-      <c r="C40" s="42"/>
-      <c r="D40" s="39"/>
-      <c r="E40" s="7"/>
-      <c r="F40" s="45"/>
-      <c r="G40" s="26"/>
-      <c r="H40" s="7"/>
-      <c r="I40" s="33"/>
-    </row>
-    <row r="41" spans="1:9" ht="21.75" x14ac:dyDescent="0.2">
-      <c r="A41" s="33"/>
-      <c r="B41" s="33"/>
-      <c r="C41" s="42"/>
-      <c r="D41" s="39"/>
-      <c r="E41" s="7"/>
-      <c r="F41" s="45"/>
-      <c r="G41" s="26"/>
-      <c r="H41" s="7"/>
-      <c r="I41" s="33"/>
-    </row>
-    <row r="42" spans="1:9" ht="21.75" x14ac:dyDescent="0.2">
-      <c r="A42" s="33"/>
-      <c r="B42" s="33"/>
-      <c r="C42" s="42"/>
-      <c r="D42" s="39"/>
-      <c r="E42" s="7"/>
-      <c r="F42" s="45"/>
-      <c r="G42" s="26"/>
-      <c r="H42" s="7"/>
-      <c r="I42" s="33"/>
-    </row>
-    <row r="43" spans="1:9" ht="22.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="34"/>
-      <c r="B43" s="34"/>
-      <c r="C43" s="43"/>
-      <c r="D43" s="40"/>
-      <c r="E43" s="14"/>
-      <c r="F43" s="46"/>
-      <c r="G43" s="27"/>
-      <c r="H43" s="14"/>
-      <c r="I43" s="34"/>
-    </row>
-    <row r="44" spans="1:9" ht="22.5" thickTop="1" x14ac:dyDescent="0.2">
-      <c r="A44" s="32" t="s">
-        <v>22</v>
-      </c>
-      <c r="B44" s="32" t="s">
-        <v>31</v>
-      </c>
-      <c r="C44" s="44">
-        <v>0</v>
-      </c>
-      <c r="D44" s="38"/>
-      <c r="E44" s="15"/>
-      <c r="F44" s="47"/>
-      <c r="G44" s="28"/>
-      <c r="H44" s="15"/>
-      <c r="I44" s="32"/>
-    </row>
-    <row r="45" spans="1:9" ht="21.75" x14ac:dyDescent="0.2">
-      <c r="A45" s="33"/>
-      <c r="B45" s="33"/>
-      <c r="C45" s="42"/>
-      <c r="D45" s="39"/>
-      <c r="E45" s="7"/>
-      <c r="F45" s="45"/>
-      <c r="G45" s="26"/>
-      <c r="H45" s="7"/>
-      <c r="I45" s="33"/>
-    </row>
-    <row r="46" spans="1:9" ht="21.75" x14ac:dyDescent="0.2">
-      <c r="A46" s="33"/>
-      <c r="B46" s="33"/>
-      <c r="C46" s="42"/>
-      <c r="D46" s="39"/>
-      <c r="E46" s="7"/>
-      <c r="F46" s="45"/>
-      <c r="G46" s="26"/>
-      <c r="H46" s="7"/>
-      <c r="I46" s="33"/>
-    </row>
-    <row r="47" spans="1:9" ht="21.75" x14ac:dyDescent="0.2">
-      <c r="A47" s="33"/>
-      <c r="B47" s="33"/>
-      <c r="C47" s="42"/>
-      <c r="D47" s="39"/>
-      <c r="E47" s="7"/>
-      <c r="F47" s="45"/>
-      <c r="G47" s="26"/>
-      <c r="H47" s="7"/>
-      <c r="I47" s="33"/>
-    </row>
-    <row r="48" spans="1:9" ht="21.75" x14ac:dyDescent="0.2">
-      <c r="A48" s="33"/>
-      <c r="B48" s="33"/>
-      <c r="C48" s="42"/>
-      <c r="D48" s="39"/>
-      <c r="E48" s="7"/>
-      <c r="F48" s="45"/>
-      <c r="G48" s="26"/>
-      <c r="H48" s="7"/>
-      <c r="I48" s="33"/>
-    </row>
-    <row r="49" spans="1:9" ht="22.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="34"/>
-      <c r="B49" s="34"/>
-      <c r="C49" s="43"/>
-      <c r="D49" s="40"/>
-      <c r="E49" s="14"/>
-      <c r="F49" s="46"/>
-      <c r="G49" s="27"/>
-      <c r="H49" s="14"/>
-      <c r="I49" s="34"/>
-    </row>
-    <row r="50" spans="1:9" ht="66.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.2">
-      <c r="A50" s="23" t="s">
-        <v>23</v>
-      </c>
-      <c r="B50" s="24"/>
-      <c r="C50" s="19">
+      <c r="B50" s="35"/>
+      <c r="C50" s="16">
         <f>SUM(C8:C49)</f>
         <v>0</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="51">
+  <mergeCells count="49">
+    <mergeCell ref="A50:B50"/>
+    <mergeCell ref="G8:G13"/>
+    <mergeCell ref="G14:G19"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="A14:A19"/>
+    <mergeCell ref="B14:B19"/>
+    <mergeCell ref="C14:C19"/>
+    <mergeCell ref="D14:D19"/>
+    <mergeCell ref="I14:I19"/>
+    <mergeCell ref="E6:F6"/>
+    <mergeCell ref="D8:D13"/>
+    <mergeCell ref="C8:C13"/>
+    <mergeCell ref="B8:B13"/>
+    <mergeCell ref="A8:A13"/>
+    <mergeCell ref="I8:I13"/>
+    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="A20:A25"/>
+    <mergeCell ref="B20:B25"/>
+    <mergeCell ref="C20:C25"/>
+    <mergeCell ref="D20:D25"/>
+    <mergeCell ref="G20:G25"/>
+    <mergeCell ref="I20:I25"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="A5:B5"/>
+    <mergeCell ref="B32:B37"/>
+    <mergeCell ref="C32:C37"/>
+    <mergeCell ref="D32:D37"/>
+    <mergeCell ref="G32:G37"/>
+    <mergeCell ref="A26:A31"/>
+    <mergeCell ref="B26:B31"/>
+    <mergeCell ref="C26:C31"/>
+    <mergeCell ref="D26:D31"/>
+    <mergeCell ref="G26:G31"/>
     <mergeCell ref="A2:B2"/>
     <mergeCell ref="I44:I49"/>
     <mergeCell ref="A44:A49"/>
@@ -1523,41 +1556,6 @@
     <mergeCell ref="G38:G43"/>
     <mergeCell ref="I38:I43"/>
     <mergeCell ref="A32:A37"/>
-    <mergeCell ref="B32:B37"/>
-    <mergeCell ref="C32:C37"/>
-    <mergeCell ref="D32:D37"/>
-    <mergeCell ref="G32:G37"/>
-    <mergeCell ref="A26:A31"/>
-    <mergeCell ref="B26:B31"/>
-    <mergeCell ref="C26:C31"/>
-    <mergeCell ref="D26:D31"/>
-    <mergeCell ref="G26:G31"/>
-    <mergeCell ref="A8:A13"/>
-    <mergeCell ref="I8:I13"/>
-    <mergeCell ref="A3:B3"/>
-    <mergeCell ref="A20:A25"/>
-    <mergeCell ref="B20:B25"/>
-    <mergeCell ref="C20:C25"/>
-    <mergeCell ref="D20:D25"/>
-    <mergeCell ref="G20:G25"/>
-    <mergeCell ref="I20:I25"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="A5:B5"/>
-    <mergeCell ref="A50:B50"/>
-    <mergeCell ref="G8:G13"/>
-    <mergeCell ref="G14:G19"/>
-    <mergeCell ref="C1:I1"/>
-    <mergeCell ref="C3:I3"/>
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="A14:A19"/>
-    <mergeCell ref="B14:B19"/>
-    <mergeCell ref="C14:C19"/>
-    <mergeCell ref="D14:D19"/>
-    <mergeCell ref="I14:I19"/>
-    <mergeCell ref="E6:F6"/>
-    <mergeCell ref="D8:D13"/>
-    <mergeCell ref="C8:C13"/>
-    <mergeCell ref="B8:B13"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -1565,23 +1563,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="b0813688-1b74-449d-9314-201dc0daaba4" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101003AFBAE34FB22D147B9C07CA883E56CB7" ma:contentTypeVersion="15" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="71f01b2d7ceacc06b6a052d001823ce1">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="0b1e59f7-8d47-4ce3-916d-39ae99b0dcd8" xmlns:ns4="b0813688-1b74-449d-9314-201dc0daaba4" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="fb427d3e1bd774699394e3b06b8fea32" ns3:_="" ns4:_="">
     <xsd:import namespace="0b1e59f7-8d47-4ce3-916d-39ae99b0dcd8"/>
@@ -1814,32 +1795,24 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F2D22B06-8882-4005-A543-0F1B8DD25376}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="0b1e59f7-8d47-4ce3-916d-39ae99b0dcd8"/>
-    <ds:schemaRef ds:uri="b0813688-1b74-449d-9314-201dc0daaba4"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4C7E44F4-C776-4F77-B375-B421E9598698}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="b0813688-1b74-449d-9314-201dc0daaba4" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6ED0CC49-9D29-4426-ACCC-E59442520F85}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1856,4 +1829,29 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4C7E44F4-C776-4F77-B375-B421E9598698}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F2D22B06-8882-4005-A543-0F1B8DD25376}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="0b1e59f7-8d47-4ce3-916d-39ae99b0dcd8"/>
+    <ds:schemaRef ds:uri="b0813688-1b74-449d-9314-201dc0daaba4"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>